<commit_message>
fix: select branch courts from live options and test HUG samples
</commit_message>
<xml_diff>
--- a/court-search/test_input.xlsx
+++ b/court-search/test_input.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="조회대상" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,168 +413,108 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>법원</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>사건번호</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>비고</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>당사자명</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>출처URL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>전주지방법원</t>
+          <t>홍성지원</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2024타인1057</t>
+          <t>2024타인108</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>국가법령정보센터 판례</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>주택</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://www.law.go.kr/DRF/lawService.do?ID=606803&amp;OC=unicpla&amp;mobileYn=Y&amp;target=prec&amp;type=HTML</t>
+          <t>주택도시보증공사</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>청주지방법원</t>
+          <t>홍성지원</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2019타인269</t>
+          <t>2024타인109</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>국가법령정보센터 판례</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>주택</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://law.go.kr/LSW/precInfoP.do?precSeq=223301</t>
+          <t>주택도시보증공사</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>서울북부지방법원</t>
+          <t>서울남부지방법원</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2018타인389</t>
+          <t>2024타인220</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>세종사이버대학교 자료</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>주택</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://home.sjcu.ac.kr/realty/community/data.do?articleNo=63330&amp;attachNo=24180&amp;mode=download</t>
+          <t>주택도시보증공사</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>부산지방법원</t>
+          <t>평택지원</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024타인368</t>
+          <t>2023타인84</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>가로수경매 공개자료</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>주택</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://garosuauction.com/m/search/detail_view.php?idx=1330302</t>
+          <t>주택도시보증공사</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>제주지방법원</t>
+          <t>평택지원</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024타인157</t>
+          <t>2023타인3</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>마이옥션 공개자료</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>주택</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://www.my-auction.co.kr/view3/1203559/ljs874</t>
+          <t>주택도시보증공사</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: disambiguate Hongseong district court and Pyeongtaek full name
</commit_message>
<xml_diff>
--- a/court-search/test_input.xlsx
+++ b/court-search/test_input.xlsx
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>홍성지원</t>
+          <t>대전지방법원 홍성지원</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -453,7 +453,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>홍성지원</t>
+          <t>대전지방법원 홍성지원</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -487,7 +487,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>평택지원</t>
+          <t>수원지방법원 평택지원</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>평택지원</t>
+          <t>수원지방법원 평택지원</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>